<commit_message>
Fix reskilling similarity to use z-scored Basic+Technical+Knowledge skills instead of raw Basic Skills alone, add NCES CIP-SOC field-of-study tagging with crosswalk-granularity caveat, and bring the Data Dictionary's dataset registry current
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/From_Exposure_to_Action_Data_Dictionary.xlsx
+++ b/docs/From_Exposure_to_Action_Data_Dictionary.xlsx
@@ -765,9 +765,9 @@
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="B25:F25"/>
     <mergeCell ref="B28:F28"/>
-    <mergeCell ref="B14:F14"/>
     <mergeCell ref="B23:F23"/>
     <mergeCell ref="B22:F22"/>
+    <mergeCell ref="B14:F14"/>
     <mergeCell ref="B8:F8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -914,12 +914,12 @@
       </c>
       <c r="K2" s="10" t="inlineStr">
         <is>
-          <t>Not yet pulled</t>
+          <t>Pulled</t>
         </is>
       </c>
       <c r="L2" s="10" t="inlineStr">
         <is>
-          <t>Free academic use; cite Felten, Raj &amp; Seamans (2021), Strategic Management Journal.</t>
+          <t>Pulled via fetch_aioe.py from the authors' own GitHub repo (AIOE_DataAppendix.xlsx, Appendix A), keyed by 6-digit SOC code (774 occupations). Note: the published AIOE index is already a standardized (z-scored) value, mean 0 / SD 1 -- not a raw score. Used directly as aioe_score in the master table and as one input to composite_exposure_score.</t>
         </is>
       </c>
     </row>
@@ -976,12 +976,12 @@
       </c>
       <c r="K3" s="11" t="inlineStr">
         <is>
-          <t>Not yet pulled</t>
+          <t>Dropped</t>
         </is>
       </c>
       <c r="L3" s="11" t="inlineStr">
         <is>
-          <t>Newest/most methodologically rigorous exposure index; measures proximity of AI capability to job needs, not just 'can AI do this.'</t>
+          <t>Investigated and dropped -- confirmed (not assumed) that OECD has never actually published the occupation-level dataset the paper (AI Papers No. 59) claims exists. fetch_oecd_exposure.py downloads the 60-page PDF report itself (O*NET-SOC-keyed, per the paper's own text), but checked oecd.ai, oecd.org, OECD iLibrary, the Data Explorer, and GitHub -- no downloadable xlsx/csv exists anywhere. A confirmed dead end, not a pending item; see src/data_acquisition/README.md.</t>
         </is>
       </c>
     </row>
@@ -1038,12 +1038,12 @@
       </c>
       <c r="K4" s="10" t="inlineStr">
         <is>
-          <t>Not yet pulled</t>
+          <t>Pulled</t>
         </is>
       </c>
       <c r="L4" s="10" t="inlineStr">
         <is>
-          <t>ILO explicitly warns exposure is not the same as a job-loss forecast — cite this caveat in the final report.</t>
+          <t>Pulled via fetch_ilo_genai.py from the lead author's own GitHub repo. Final_Scores_ISCO08_Gmyrek_et_al_2025.xlsx is actually stored at task granularity but carries pre-aggregated mean_score_2025/SD_2025 per ISCO-08 occupation (427 occupations); 4digits_with_tasks.xlsx turned out to hold only categorical exposure labels, not a numeric score, so it is downloaded but not used. Mapped ISCO-08 -&gt; SOC 2018 via the chained BLS crosswalks (see BLS OEWS row). Feeds ilo_score, ilo_task_mean/std, and the provisional impact_pattern classification (840 SOC occupations after crosswalk aggregation).</t>
         </is>
       </c>
     </row>
@@ -1100,12 +1100,12 @@
       </c>
       <c r="K5" s="11" t="inlineStr">
         <is>
-          <t>Not yet pulled</t>
+          <t>Pulled</t>
         </is>
       </c>
       <c r="L5" s="11" t="inlineStr">
         <is>
-          <t>Job Zones file gives required education/experience/training per occupation — this is the key student-facing join.</t>
+          <t>Job Zones file gives required education/experience/training per occupation — this is the key student-facing join. Pulled and integrated: Occupation Data (SOC crosswalk), Job Zones, Essential Skills (10 Basic Skills, skill__* columns), Transferable Skills (24 Cross-Functional skills, xfskill__* columns), and Knowledge (33 domains, knowledge__* columns). Not yet pulled: Abilities.xlsx and Work Activities.xlsx (both already downloaded to data/raw/ but not yet loaded into the master table).</t>
         </is>
       </c>
     </row>
@@ -1162,12 +1162,12 @@
       </c>
       <c r="K6" s="10" t="inlineStr">
         <is>
-          <t>Not yet pulled</t>
+          <t>Pulled</t>
         </is>
       </c>
       <c r="L6" s="10" t="inlineStr">
         <is>
-          <t>Pull multiple years (not just one) to build the panel needed for a trend comparison. Only historical/descriptive — not a forecast.</t>
+          <t>Pulled via fetch_bls_oews.py -- bls.gov blocks scripted downloads at the WAF level (same block as the BLS SOC crosswalks), so the 3 years of national "All Data" tables (oesm23nat/24nat/25nat.zip) were downloaded manually and placed in data/raw/; the script picks them up automatically once present. load_bls_oews_growth() reduces each year to one economy-wide, detailed-occupation row per SOC code and computes employment_growth_rate as the annualized (CAGR) change 2023-&gt;2025 -- integrated into the master table (831 SOC occupations). Optional at merge_all() time: if fewer than 2 years are present, this column is simply absent rather than the run failing.</t>
         </is>
       </c>
     </row>
@@ -1224,12 +1224,12 @@
       </c>
       <c r="K7" s="11" t="inlineStr">
         <is>
-          <t>Not yet pulled</t>
+          <t>Pulled</t>
         </is>
       </c>
       <c r="L7" s="11" t="inlineStr">
         <is>
-          <t>One of the most-cited LLM-specific exposure measures; good robustness check against AIOE/OECD.</t>
+          <t>Pulled via fetch_gpts_are_gpts.py from the authors' own openai/GPTs-are-GPTs GitHub repo (occ_level.csv), keyed by O*NET-SOC Code (923 occupations). Uses dv_rating_beta (GPT-4-generated label) as gpts_are_gpts_score, consistent with AIOE/ILO as an automated/model-based measure; human_rating_beta -- confirmed against the paper's own text to be its actual headline measure (the 80%/19% worker statistics) -- is kept alongside as gpts_are_gpts_human_score for correct citation and cross-check.</t>
         </is>
       </c>
     </row>
@@ -1286,12 +1286,12 @@
       </c>
       <c r="K8" s="10" t="inlineStr">
         <is>
-          <t>Not yet pulled</t>
+          <t>Partially pulled</t>
         </is>
       </c>
       <c r="L8" s="10" t="inlineStr">
         <is>
-          <t>Measures actual usage, a different concept from exposure/capability — keep as a separate variable, not merged into the composite exposure index.</t>
+          <t>Pulled via fetch_anthropic_economic_index.py from Anthropic's own Hugging Face repo, latest release as of this project (2026-06-26). Both the 1P API and claude.ai usage CSVs are downloaded, but only the 1P API release is integrated into the master table (anthropic_1p_automation_share / anthropic_1p_augmentation_share, global-only and unambiguous) -- the richer claude.ai release has per-country breakdowns and multiple occupation hierarchy levels whose global-aggregate row is not yet confirmed, so it remains unintegrated. Real usage evidence, kept separate from composite_exposure_score.</t>
         </is>
       </c>
     </row>
@@ -1348,12 +1348,12 @@
       </c>
       <c r="K9" s="11" t="inlineStr">
         <is>
-          <t>Not yet pulled</t>
+          <t>Pulled (appendix only)</t>
         </is>
       </c>
       <c r="L9" s="11" t="inlineStr">
         <is>
-          <t>Official, NOC-native — no crosswalk needed for this one specifically.</t>
+          <t>Pulled via fetch_statcan_canada.py -- saves the source article page (Mehdi &amp; Morissette 2024, Statistics Canada, Sept 3 2024) since no separate data file exists. load_statcan_noc_exposure() parses Appendix Table A.2 (28 NOC occupation groups, May 2021) from the saved page. Deliberately NOT joined onto the SOC-keyed master table (NOC-keyed, appendix-only per this project's guardrails) -- feeds one standalone Canada comparison chart in the notebook. Caution: StatCan recomputed AIOE themselves on their own raw scale (median ~6.0), not the z-scored value this project's own aioe_score uses -- the two must be standardized before any comparison.</t>
         </is>
       </c>
     </row>
@@ -1594,9 +1594,6 @@
           <t>No crosswalk is perfectly 1:1 — some occupations split or merge across systems. Keep the original code from each source as its own column in the master dataset rather than forcing a single unified code; this preserves traceability and lets you re-run the join if a mapping is revised.</t>
         </is>
       </c>
-      <c r="C9" s="14" t="n"/>
-      <c r="D9" s="14" t="n"/>
-      <c r="E9" s="14" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:E7"/>
@@ -2380,7 +2377,6 @@
           <t>This tab is a specification only. Do not start building it until the Phase 1 notebook/report has produced the Composite Exposure Score, Impact Pattern, and skill-similarity outputs it depends on. Every screen presents evidence and options — never a single prescriptive recommendation (see 'Guiding principle' on the Read Me tab).</t>
         </is>
       </c>
-      <c r="C16" s="14" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:C14"/>

</xml_diff>